<commit_message>
Enhance tariff import functionality and update PHPUnit configuration
- Updated `phpunit.xml` to enforce environment variable values for testing, ensuring consistent test behavior.
- Refactored `OzonTariffSheetParser` to improve header row detection and column mapping, adding new methods for better clarity and maintainability.
- Enhanced `YandexTariffSheetParser` to support parsing of parameter tables and improved error handling for channel rates.
- Introduced new methods in `CellValueNormalizer` for parsing leading decimals and handling weight ranges with spaces, improving data accuracy.
- Added comprehensive tests for the new parsing logic and updated existing tests to cover edge cases in tariff calculations.
- Included a new test suite for customer calculator cases, validating expected costs against various payloads.
- Updated documentation to reflect changes in XLSX import format and parsing rules.
</commit_message>
<xml_diff>
--- a/tests/Fixtures/xlsx/invalid-broken-rate.xlsx
+++ b/tests/Fixtures/xlsx/invalid-broken-rate.xlsx
@@ -16,39 +16,48 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="56">
-  <si>
-    <t>Channel</t>
-  </si>
-  <si>
-    <t>Weight g</t>
-  </si>
-  <si>
-    <t>Rate</t>
-  </si>
-  <si>
-    <t>Limits</t>
-  </si>
-  <si>
-    <t>Order CNY</t>
-  </si>
-  <si>
-    <t>Order RUB</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="60">
+  <si>
+    <t>Delivery Method</t>
+  </si>
+  <si>
+    <t>Rates (PUDO / Courier)</t>
+  </si>
+  <si>
+    <t>Measurements, max cm</t>
+  </si>
+  <si>
+    <t>Shipment weight limits / min g</t>
+  </si>
+  <si>
+    <t>Shipment weight limits / max g</t>
+  </si>
+  <si>
+    <t>Shipment cost limit / min-max  | RUB</t>
+  </si>
+  <si>
+    <t>Shipment cost limit / min-max  | CNY</t>
+  </si>
+  <si>
+    <t>Tarification type</t>
   </si>
   <si>
     <t>ATC Express Extra Small</t>
   </si>
   <si>
+    <t>¥ 3.37 + ¥ 0.0505/1 g</t>
+  </si>
+  <si>
+    <t>Sum of sides ≤ 90 cm, length ≤ 60 cm</t>
+  </si>
+  <si>
     <t>1 - 1500</t>
   </si>
   <si>
-    <t>¥ 4.10 + ¥ 0.0600/1 g</t>
-  </si>
-  <si>
-    <t>Sum of sides ≤ 90 cm, length ≤ 60 cm</t>
-  </si>
-  <si>
-    <t>100.00 - 700.00</t>
+    <t>0.01 - 135</t>
+  </si>
+  <si>
+    <t>Physical weight</t>
   </si>
   <si>
     <t>ATC Standard Extra Small</t>
@@ -57,133 +66,136 @@
     <t>broken rate value</t>
   </si>
   <si>
-    <t>135.01 - 635.00</t>
-  </si>
-  <si>
     <t>ATC Economy Extra Small</t>
   </si>
   <si>
-    <t>¥ 2.90 + ¥ 0.0400/1 g</t>
-  </si>
-  <si>
-    <t>100.00 - 600.00</t>
+    <t>¥ 3.37 + ¥ 0.0281/1 g</t>
   </si>
   <si>
     <t>ATC Standard Budget</t>
   </si>
   <si>
-    <t>1 - 2000</t>
-  </si>
-  <si>
-    <t>¥ 2.50 + ¥ 0.0350/1 g</t>
-  </si>
-  <si>
-    <t>Sum of sides ≤ 100 cm, length ≤ 70 cm</t>
-  </si>
-  <si>
-    <t>50.00 - 500.00</t>
+    <t>¥ 25.83 + ¥ 0.0281/1 g</t>
+  </si>
+  <si>
+    <t>Sum of sides ≤ 150 cm, length ≤ 60 cm</t>
   </si>
   <si>
     <t>ATC Economy Budget</t>
   </si>
   <si>
-    <t>¥ 2.10 + ¥ 0.0300/1 g</t>
+    <t>¥ 25.83 + ¥ 0.0191/1 g</t>
   </si>
   <si>
     <t>ATC Express Small</t>
   </si>
   <si>
-    <t>1 - 5000</t>
-  </si>
-  <si>
-    <t>¥ 8.00 + ¥ 0.0450/1 g</t>
-  </si>
-  <si>
-    <t>Sum of sides ≤ 120 cm, length ≤ 80 cm</t>
-  </si>
-  <si>
-    <t>100.00 - 1500.00</t>
+    <t>¥ 17.97 + ¥ 0.0505/1 g</t>
+  </si>
+  <si>
+    <t>1501 - 7000</t>
+  </si>
+  <si>
+    <t>135.01 - 635</t>
   </si>
   <si>
     <t>ATC Standard Small</t>
   </si>
   <si>
-    <t>¥ 6.50 + ¥ 0.0380/1 g</t>
+    <t>¥ 17.97 + ¥ 0.0393/1 g</t>
   </si>
   <si>
     <t>ATC Economy Small</t>
   </si>
   <si>
-    <t>¥ 5.20 + ¥ 0.0320/1 g</t>
+    <t>¥ 17.97 + ¥ 0.0281/1 g</t>
   </si>
   <si>
     <t>ATC Standard Big</t>
   </si>
   <si>
-    <t>1 - 30000</t>
-  </si>
-  <si>
     <t>¥ 40.44 + ¥ 0.0281/1 g</t>
   </si>
   <si>
-    <t>Sum of sides ≤ 150 cm, length ≤ 100 cm</t>
+    <t>Sum of sides ≤ 310 cm, length ≤ 150 cm</t>
+  </si>
+  <si>
+    <t>Max weight between the physical and volume ones</t>
   </si>
   <si>
     <t>ATC Economy Big</t>
   </si>
   <si>
-    <t>¥ 35.00 + ¥ 0.0250/1 g</t>
+    <t>¥ 40.44 + ¥ 0.0191/1 g</t>
   </si>
   <si>
     <t>ATC Express Premium Small</t>
   </si>
   <si>
-    <t>¥ 12.00 + ¥ 0.0550/1 g</t>
-  </si>
-  <si>
-    <t>200.00 - 2000.00</t>
+    <t>¥ 24.71 + ¥ 0.0505/1 g</t>
+  </si>
+  <si>
+    <t>Sum of sides ≤ 250 cm, length ≤ 150 cm.</t>
+  </si>
+  <si>
+    <t>7001 - 250000</t>
+  </si>
+  <si>
+    <t>635.01 - 22525</t>
   </si>
   <si>
     <t>ATC Standard Premium Small</t>
   </si>
   <si>
-    <t>¥ 10.00 + ¥ 0.0480/1 g</t>
+    <t>¥ 24.71 + ¥ 0.0393/1 g</t>
   </si>
   <si>
     <t>ATC Economy Premium Small</t>
   </si>
   <si>
-    <t>¥ 8.50 + ¥ 0.0420/1 g</t>
+    <t>¥ 24.71 + ¥ 0.0281/1 g</t>
   </si>
   <si>
     <t>ATC Standard Premium Big</t>
   </si>
   <si>
-    <t>¥ 50.00 + ¥ 0.0300/1 g</t>
-  </si>
-  <si>
-    <t>Sum of sides ≤ 160 cm, length ≤ 110 cm</t>
+    <t>¥ 69.64 + ¥ 0.0314/1 g</t>
   </si>
   <si>
     <t>ATC Economy Premium Big</t>
   </si>
   <si>
-    <t>¥ 45.00 + ¥ 0.0270/1 g</t>
+    <t>¥ 69.64 + ¥ 0.0258/1 g</t>
   </si>
   <si>
     <t>Yandex Market</t>
   </si>
   <si>
-    <t>Super Express 空运卡航</t>
-  </si>
-  <si>
-    <t>193 + 948 RUB/kg</t>
-  </si>
-  <si>
-    <t>Express 卡航陆运</t>
-  </si>
-  <si>
-    <t>198 RUB + 787 /kg</t>
+    <t>Параметр</t>
+  </si>
+  <si>
+    <t>Super Express (空运卡航)</t>
+  </si>
+  <si>
+    <t>Express (卡航陆运)</t>
+  </si>
+  <si>
+    <t>Ставка за кг</t>
+  </si>
+  <si>
+    <t>948 ₽/кг</t>
+  </si>
+  <si>
+    <t>787 ₽/кг</t>
+  </si>
+  <si>
+    <t>Фиксированная ставка за заказ</t>
+  </si>
+  <si>
+    <t>193 ₽/шт</t>
+  </si>
+  <si>
+    <t>198 ₽/шт</t>
   </si>
 </sst>
 </file>
@@ -523,10 +535,10 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:8">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -545,248 +557,401 @@
       <c r="F1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:6">
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8">
       <c r="A2" t="s">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D2" t="s">
-        <v>9</v>
-      </c>
-      <c r="E2" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="3" spans="1:6">
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2">
+        <v>500</v>
+      </c>
+      <c r="F2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G2" t="s">
+        <v>12</v>
+      </c>
+      <c r="H2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8">
       <c r="A3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="E3">
+        <v>500</v>
+      </c>
+      <c r="F3" t="s">
         <v>11</v>
       </c>
-      <c r="B3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C3" t="s">
+      <c r="G3" t="s">
         <v>12</v>
       </c>
-      <c r="D3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E3" t="s">
+      <c r="H3" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:8">
       <c r="A4" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B4" t="s">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="C4" t="s">
-        <v>15</v>
-      </c>
-      <c r="D4" t="s">
-        <v>9</v>
-      </c>
-      <c r="E4" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6">
+        <v>10</v>
+      </c>
+      <c r="D4">
+        <v>1</v>
+      </c>
+      <c r="E4">
+        <v>500</v>
+      </c>
+      <c r="F4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G4" t="s">
+        <v>12</v>
+      </c>
+      <c r="H4" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8">
       <c r="A5" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B5" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C5" t="s">
-        <v>19</v>
-      </c>
-      <c r="D5" t="s">
         <v>20</v>
       </c>
-      <c r="E5" t="s">
+      <c r="D5">
+        <v>501</v>
+      </c>
+      <c r="E5">
+        <v>30000</v>
+      </c>
+      <c r="F5" t="s">
+        <v>11</v>
+      </c>
+      <c r="G5" t="s">
+        <v>12</v>
+      </c>
+      <c r="H5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8">
+      <c r="A6" t="s">
         <v>21</v>
       </c>
-    </row>
-    <row r="6" spans="1:6">
-      <c r="A6" t="s">
+      <c r="B6" t="s">
         <v>22</v>
       </c>
-      <c r="B6" t="s">
-        <v>18</v>
-      </c>
       <c r="C6" t="s">
+        <v>20</v>
+      </c>
+      <c r="D6">
+        <v>501</v>
+      </c>
+      <c r="E6">
+        <v>30000</v>
+      </c>
+      <c r="F6" t="s">
+        <v>11</v>
+      </c>
+      <c r="G6" t="s">
+        <v>12</v>
+      </c>
+      <c r="H6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8">
+      <c r="A7" t="s">
         <v>23</v>
       </c>
-      <c r="D6" t="s">
+      <c r="B7" t="s">
+        <v>24</v>
+      </c>
+      <c r="C7" t="s">
         <v>20</v>
       </c>
-      <c r="E6" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6">
-      <c r="A7" t="s">
-        <v>24</v>
-      </c>
-      <c r="B7" t="s">
+      <c r="D7">
+        <v>1</v>
+      </c>
+      <c r="E7">
+        <v>2000</v>
+      </c>
+      <c r="F7" t="s">
         <v>25</v>
       </c>
-      <c r="C7" t="s">
+      <c r="G7" t="s">
         <v>26</v>
       </c>
-      <c r="D7" t="s">
+      <c r="H7" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8">
+      <c r="A8" t="s">
         <v>27</v>
       </c>
-      <c r="E7" t="s">
+      <c r="B8" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="8" spans="1:6">
-      <c r="A8" t="s">
+      <c r="C8" t="s">
+        <v>20</v>
+      </c>
+      <c r="D8">
+        <v>1</v>
+      </c>
+      <c r="E8">
+        <v>2000</v>
+      </c>
+      <c r="F8" t="s">
+        <v>25</v>
+      </c>
+      <c r="G8" t="s">
+        <v>26</v>
+      </c>
+      <c r="H8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8">
+      <c r="A9" t="s">
         <v>29</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B9" t="s">
+        <v>30</v>
+      </c>
+      <c r="C9" t="s">
+        <v>20</v>
+      </c>
+      <c r="D9">
+        <v>1</v>
+      </c>
+      <c r="E9">
+        <v>2000</v>
+      </c>
+      <c r="F9" t="s">
         <v>25</v>
       </c>
-      <c r="C8" t="s">
-        <v>30</v>
-      </c>
-      <c r="D8" t="s">
-        <v>27</v>
-      </c>
-      <c r="E8" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6">
-      <c r="A9" t="s">
+      <c r="G9" t="s">
+        <v>26</v>
+      </c>
+      <c r="H9" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8">
+      <c r="A10" t="s">
         <v>31</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B10" t="s">
+        <v>32</v>
+      </c>
+      <c r="C10" t="s">
+        <v>33</v>
+      </c>
+      <c r="D10">
+        <v>2001</v>
+      </c>
+      <c r="E10">
+        <v>30000</v>
+      </c>
+      <c r="F10" t="s">
         <v>25</v>
       </c>
-      <c r="C9" t="s">
-        <v>32</v>
-      </c>
-      <c r="D9" t="s">
-        <v>27</v>
-      </c>
-      <c r="E9" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6">
-      <c r="A10" t="s">
+      <c r="G10" t="s">
+        <v>26</v>
+      </c>
+      <c r="H10" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8">
+      <c r="A11" t="s">
+        <v>35</v>
+      </c>
+      <c r="B11" t="s">
+        <v>36</v>
+      </c>
+      <c r="C11" t="s">
         <v>33</v>
       </c>
-      <c r="B10" t="s">
+      <c r="D11">
+        <v>2001</v>
+      </c>
+      <c r="E11">
+        <v>30000</v>
+      </c>
+      <c r="F11" t="s">
+        <v>25</v>
+      </c>
+      <c r="G11" t="s">
+        <v>26</v>
+      </c>
+      <c r="H11" t="s">
         <v>34</v>
       </c>
-      <c r="C10" t="s">
-        <v>35</v>
-      </c>
-      <c r="D10" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6">
-      <c r="A11" t="s">
+    </row>
+    <row r="12" spans="1:8">
+      <c r="A12" t="s">
         <v>37</v>
       </c>
-      <c r="B11" t="s">
-        <v>34</v>
-      </c>
-      <c r="C11" t="s">
+      <c r="B12" t="s">
         <v>38</v>
       </c>
-      <c r="D11" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6">
-      <c r="A12" t="s">
+      <c r="C12" t="s">
         <v>39</v>
       </c>
-      <c r="B12" t="s">
-        <v>25</v>
-      </c>
-      <c r="C12" t="s">
+      <c r="D12">
+        <v>1</v>
+      </c>
+      <c r="E12">
+        <v>5000</v>
+      </c>
+      <c r="F12" t="s">
         <v>40</v>
       </c>
-      <c r="D12" t="s">
-        <v>27</v>
-      </c>
-      <c r="E12" t="s">
+      <c r="G12" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="13" spans="1:6">
+      <c r="H12" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8">
       <c r="A13" t="s">
         <v>42</v>
       </c>
       <c r="B13" t="s">
-        <v>25</v>
+        <v>43</v>
       </c>
       <c r="C13" t="s">
-        <v>43</v>
-      </c>
-      <c r="D13" t="s">
-        <v>27</v>
-      </c>
-      <c r="E13" t="s">
+        <v>39</v>
+      </c>
+      <c r="D13">
+        <v>1</v>
+      </c>
+      <c r="E13">
+        <v>5000</v>
+      </c>
+      <c r="F13" t="s">
+        <v>40</v>
+      </c>
+      <c r="G13" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="14" spans="1:6">
+      <c r="H13" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8">
       <c r="A14" t="s">
         <v>44</v>
       </c>
       <c r="B14" t="s">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="C14" t="s">
-        <v>45</v>
-      </c>
-      <c r="D14" t="s">
-        <v>27</v>
-      </c>
-      <c r="E14" t="s">
+        <v>39</v>
+      </c>
+      <c r="D14">
+        <v>1</v>
+      </c>
+      <c r="E14">
+        <v>5000</v>
+      </c>
+      <c r="F14" t="s">
+        <v>40</v>
+      </c>
+      <c r="G14" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="15" spans="1:6">
+      <c r="H14" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8">
       <c r="A15" t="s">
         <v>46</v>
       </c>
       <c r="B15" t="s">
+        <v>47</v>
+      </c>
+      <c r="C15" t="s">
+        <v>33</v>
+      </c>
+      <c r="D15">
+        <v>5001</v>
+      </c>
+      <c r="E15">
+        <v>30000</v>
+      </c>
+      <c r="F15" t="s">
+        <v>40</v>
+      </c>
+      <c r="G15" t="s">
+        <v>41</v>
+      </c>
+      <c r="H15" t="s">
         <v>34</v>
       </c>
-      <c r="C15" t="s">
-        <v>47</v>
-      </c>
-      <c r="D15" t="s">
+    </row>
+    <row r="16" spans="1:8">
+      <c r="A16" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="16" spans="1:6">
-      <c r="A16" t="s">
+      <c r="B16" t="s">
         <v>49</v>
       </c>
-      <c r="B16" t="s">
+      <c r="C16" t="s">
+        <v>33</v>
+      </c>
+      <c r="D16">
+        <v>5001</v>
+      </c>
+      <c r="E16">
+        <v>30000</v>
+      </c>
+      <c r="F16" t="s">
+        <v>40</v>
+      </c>
+      <c r="G16" t="s">
+        <v>41</v>
+      </c>
+      <c r="H16" t="s">
         <v>34</v>
-      </c>
-      <c r="C16" t="s">
-        <v>50</v>
-      </c>
-      <c r="D16" t="s">
-        <v>48</v>
       </c>
     </row>
   </sheetData>
@@ -801,36 +966,45 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:3">
       <c r="A1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
         <v>51</v>
       </c>
-    </row>
-    <row r="2" spans="1:2">
-      <c r="A2" t="s">
-        <v>0</v>
-      </c>
       <c r="B2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2">
+        <v>52</v>
+      </c>
+      <c r="C2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B3" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2">
+        <v>55</v>
+      </c>
+      <c r="C3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="B4" t="s">
-        <v>55</v>
+        <v>58</v>
+      </c>
+      <c r="C4" t="s">
+        <v>59</v>
       </c>
     </row>
   </sheetData>

</xml_diff>